<commit_message>
Finish implement phase 1.1
</commit_message>
<xml_diff>
--- a/RougeSnake_Implementation_Tracker.xlsx
+++ b/RougeSnake_Implementation_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GameProj\RougeSnake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2DDC86-BBDB-49AF-801E-5E2D019C7A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E80A46-314A-4B01-B745-80018872450C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1095" yWindow="1950" windowWidth="37305" windowHeight="14250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="185">
   <si>
     <t>Phase</t>
   </si>
@@ -587,9 +587,6 @@
   </si>
   <si>
     <t>Discuss architecture → user implements C++ → review uploaded source → playtest → lock feature.</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>Done</t>
@@ -1275,7 +1272,7 @@
         <v>2</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>12</v>
@@ -2412,7 +2409,7 @@
       </c>
       <c r="B6" s="3">
         <f>COUNTIF('Implementation Plan'!E2:E35,"Done")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
Adding render+ spawn room from json
</commit_message>
<xml_diff>
--- a/RougeSnake_Implementation_Tracker.xlsx
+++ b/RougeSnake_Implementation_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GameProj\RougeSnake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0E80A46-314A-4B01-B745-80018872450C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B45BF8-D714-4BCE-B807-6F2146675813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1095" yWindow="1950" windowWidth="37305" windowHeight="14250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="186">
   <si>
     <t>Phase</t>
   </si>
@@ -590,6 +590,9 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1333,7 @@
         <v>2</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>12</v>
@@ -1359,7 +1362,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>11</v>
+        <v>185</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>12</v>
@@ -2409,7 +2412,7 @@
       </c>
       <c r="B6" s="3">
         <f>COUNTIF('Implementation Plan'!E2:E35,"Done")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
implement phase 3 + improve code
</commit_message>
<xml_diff>
--- a/RougeSnake_Implementation_Tracker.xlsx
+++ b/RougeSnake_Implementation_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GameProj\RougeSnake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B45BF8-D714-4BCE-B807-6F2146675813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BF9F30-50FC-43E1-A68E-6976A8A51428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1095" yWindow="1950" windowWidth="37305" windowHeight="14250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Implementation Plan" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="185">
   <si>
     <t>Phase</t>
   </si>
@@ -590,9 +590,6 @@
   </si>
   <si>
     <t>Done</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -1362,7 +1359,7 @@
         <v>3</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F5" s="4" t="s">
         <v>12</v>
@@ -1391,7 +1388,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>12</v>
@@ -1420,7 +1417,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>12</v>
@@ -1449,7 +1446,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>12</v>
@@ -2412,7 +2409,7 @@
       </c>
       <c r="B6" s="3">
         <f>COUNTIF('Implementation Plan'!E2:E35,"Done")</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>

</xml_diff>

<commit_message>
Adding enemy heal + player collision
</commit_message>
<xml_diff>
--- a/RougeSnake_Implementation_Tracker.xlsx
+++ b/RougeSnake_Implementation_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\GameProj\RougeSnake\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BF9F30-50FC-43E1-A68E-6976A8A51428}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9DF07C7-E272-4A7C-84F8-9280C899B52B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="186">
   <si>
     <t>Phase</t>
   </si>
@@ -590,6 +590,9 @@
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>In Progress</t>
   </si>
 </sst>
 </file>
@@ -1475,7 +1478,7 @@
         <v>2</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>12</v>
@@ -1504,7 +1507,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>12</v>
@@ -1533,7 +1536,7 @@
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>11</v>
+        <v>184</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>12</v>
@@ -1823,7 +1826,7 @@
         <v>2</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>11</v>
+        <v>185</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>12</v>
@@ -2409,7 +2412,7 @@
       </c>
       <c r="B6" s="3">
         <f>COUNTIF('Implementation Plan'!E2:E35,"Done")</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D6" s="3">
         <v>2</v>

</xml_diff>